<commit_message>
iterate on tool annotation
</commit_message>
<xml_diff>
--- a/analysis_visualization/1.2_tools_annotated.xlsx
+++ b/analysis_visualization/1.2_tools_annotated.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2141,6 +2141,2071 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ATAE-LSTM</t>
+        </is>
+      </c>
+      <c r="B52">
+        <v>26</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>ATAE‑LSTM is an attention‑based LSTM architecture designed for aspect‑level sentiment (opinion) analysis. It can be used to measure opinions in text and is specifically built for that purpose, but it is a model architecture rather than a packaged software tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LSA</t>
+        </is>
+      </c>
+      <c r="B53">
+        <v>26</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Latent Semantic Analysis (LSA) is a statistical algorithm for extracting semantic structure from text. It can be incorporated into opinion/sentiment analysis pipelines, but it is not itself a tool specifically designed for measuring opinions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Gradient Boosting</t>
+        </is>
+      </c>
+      <c r="B54">
+        <v>25</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Gradient Boosting is a general ensemble learning algorithm that can be applied to classification tasks such as sentiment or opinion analysis, but it is not specifically designed for opinion measurement and is not itself a software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>IAN</t>
+        </is>
+      </c>
+      <c r="B55">
+        <v>25</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>other_unclear</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>The acronym "IAN" is ambiguous without additional context; it could refer to a variety of tools, frameworks, or resources, and it is not clear whether it pertains to opinion measurement or is provided as installable software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Bing Liu Opinion Lexicon</t>
+        </is>
+      </c>
+      <c r="B56">
+        <v>24</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>linguistic_resource</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>A lexical resource containing positive and negative opinion words compiled by Bing Liu, used specifically for sentiment and opinion analysis but provided as a data list rather than installable software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B57">
+        <v>23</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>programming_language</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>R is a general-purpose programming language and environment for statistical computing; it can be used to implement opinion measurement methods via packages, but the language itself is not a dedicated opinion measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>k-means</t>
+        </is>
+      </c>
+      <c r="B58">
+        <v>23</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>k-means is a general unsupervised clustering algorithm; it is not designed for extracting or measuring opinions from text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RapidMiner</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>22</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>gui_tool</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>RapidMiner is a visual data science platform with GUI-based workflows that includes text mining and sentiment analysis operators, allowing it to be used for opinion measurement but it is not dedicated solely to that purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TD-LSTM</t>
+        </is>
+      </c>
+      <c r="B60">
+        <v>22</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>TD-LSTM (Target‑Dependent LSTM) is a neural network architecture designed for aspect‑based sentiment analysis, enabling opinion measurement focused on specific targets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>doc2vec</t>
+        </is>
+      </c>
+      <c r="B61">
+        <v>22</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>doc2vec is a general algorithm for learning document embeddings; it can be used as features for opinion/sentiment analysis but is not specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Bernoulli Naive Bayes</t>
+        </is>
+      </c>
+      <c r="B62">
+        <v>21</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Bernoulli Naive Bayes is a probabilistic classification algorithm that can be applied to binary feature vectors, often used for text classification tasks such as sentiment analysis, but it is a general algorithm not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="B63">
+        <v>21</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>JST (Joint Sentiment‑Topic model) is a probabilistic algorithm that jointly models sentiment and topics for opinion mining; it can be used to measure opinions and is specifically designed for that purpose, but its availability as a reusable, installable software package is unclear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MPQA</t>
+        </is>
+      </c>
+      <c r="B64">
+        <v>21</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>linguistic_resource</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>The MPQA (Multi‑Perspective Question Answering) Opinion Corpus and associated lexicon provide annotated data for subjectivity and opinion detection, specifically designed for opinion measurement but are provided as a dataset rather than installable software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Keras</t>
+        </is>
+      </c>
+      <c r="B65">
+        <v>20</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>general_library</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Keras is a high‑level deep‑learning library for building neural network models; it can be used to create opinion/sentiment classifiers but is not specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>General Inquirer</t>
+        </is>
+      </c>
+      <c r="B66">
+        <v>19</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>linguistic_resource</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>The General Inquirer is a lexical resource that provides sentiment and other semantic categories for words, enabling opinion and sentiment analysis; it is specifically designed for opinion measurement but is a data resource rather than installable software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="B67">
+        <v>19</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Support Vector Classifier (SVC) is a machine‑learning algorithm for classification tasks; it can be employed for sentiment or opinion analysis but is not specifically designed for opinion measurement and is not a standalone software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>DBN</t>
+        </is>
+      </c>
+      <c r="B68">
+        <v>18</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>DBN (Deep Belief Network) is a neural network learning architecture that can be applied to many tasks, including sentiment or opinion analysis, but it is not a dedicated opinion‑measurement tool and is not itself a software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Gensim</t>
+        </is>
+      </c>
+      <c r="B69">
+        <v>18</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>general_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Gensim is a Python library for topic modeling, word embeddings, and similarity retrieval. It can be leveraged for opinion measurement (e.g., via sentiment‑related embeddings) but is not built specifically for that purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SMOTE</t>
+        </is>
+      </c>
+      <c r="B70">
+        <v>18</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>SMOTE (Synthetic Minority Over-sampling Technique) is a data‑augmentation algorithm for handling class imbalance; it does not extract or analyze opinions from text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Stanford Parser</t>
+        </is>
+      </c>
+      <c r="B71">
+        <v>18</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>single_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Stanford Parser is a dedicated syntactic parsing tool that produces constituency parse trees; it does not directly measure opinions, though its output can be used as a preprocessing step for opinion analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ABSA</t>
+        </is>
+      </c>
+      <c r="B72">
+        <v>17</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>approach</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>ABSA (Aspect‑Based Sentiment Analysis) is a high‑level methodology for extracting opinions about specific aspects of a target, thus it is an approach designed for opinion measurement but not a standalone software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Apache Spark</t>
+        </is>
+      </c>
+      <c r="B73">
+        <v>17</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Apache Spark is an open‑source distributed computing framework for large‑scale data processing. It can be used to run opinion‑measurement pipelines, but it does not itself provide opinion or sentiment analysis functionality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Genetic Algorithm</t>
+        </is>
+      </c>
+      <c r="B74">
+        <v>16</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Genetic Algorithm is a general optimization metaheuristic used to search for solutions in various domains; it is not a tool for extracting opinions from text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>J48</t>
+        </is>
+      </c>
+      <c r="B75">
+        <v>16</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>J48 is the implementation of the C4.5 decision‑tree algorithm (e.g., in WEKA). It is a general classification algorithm that can be applied to opinion/sentiment tasks but is not specifically designed for opinion measurement and is not itself a reusable software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>LinearSVC</t>
+        </is>
+      </c>
+      <c r="B76">
+        <v>16</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>LinearSVC is a linear support‑vector classification algorithm (often from scikit‑learn) that can be applied to sentiment or opinion classification tasks, but it is a general learning method, not a tool built specifically for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Machine Learning</t>
+        </is>
+      </c>
+      <c r="B77">
+        <v>16</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>approach</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Machine learning is a broad methodological approach for building predictive models, which can be applied to opinion/sentiment analysis but is not itself a software tool nor specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Sentiment140</t>
+        </is>
+      </c>
+      <c r="B78">
+        <v>16</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Sentiment140 provides a pre‑trained sentiment classifier (trained on 1.6 M tweets) accessible via an API, designed specifically to detect opinion polarity in short texts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Transformer</t>
+        </is>
+      </c>
+      <c r="B79">
+        <v>16</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>The Transformer is a general neural network architecture for sequence modeling; it can be employed for opinion/sentiment analysis but is not itself a dedicated opinion measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BiLSTM-CRF</t>
+        </is>
+      </c>
+      <c r="B80">
+        <v>15</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>BiLSTM-CRF is a neural network architecture (bidirectional LSTM with a CRF layer) used for sequence labeling tasks; it can be trained for opinion‑related tasks such as aspect or opinion target extraction, but it is not itself a dedicated opinion‑measurement tool and is not distributed as a standalone software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MemNet</t>
+        </is>
+      </c>
+      <c r="B81">
+        <v>15</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>MemNet (Memory Network) is a neural architecture originally proposed for tasks like sentiment analysis; it can be applied to opinion measurement and was designed with sentiment classification in mind, but it is an algorithmic model rather than a packaged software tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>OpinionFinder</t>
+        </is>
+      </c>
+      <c r="B82">
+        <v>15</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>single_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>OpinionFinder is a dedicated software system specifically designed to detect, extract, and analyze subjective language and opinions expressed in text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Word Embeddings</t>
+        </is>
+      </c>
+      <c r="B83">
+        <v>15</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>other_unclear</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Word embeddings are generic vector representations of words that can be used as features for opinion/sentiment analysis, but they are not a specific software tool, algorithm, or pre‑trained model with a concrete name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>XLNet</t>
+        </is>
+      </c>
+      <c r="B84">
+        <v>15</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>XLNet is a pre‑trained autoregressive language model that can be fine‑tuned for various NLP tasks, including sentiment or opinion analysis, but it is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>spaCy</t>
+        </is>
+      </c>
+      <c r="B85">
+        <v>15</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>general_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>spaCy is a comprehensive Python library for NLP tasks such as tokenization, parsing, and named entity recognition, and can be extended for sentiment or opinion analysis, though it is not built specifically for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ELMo</t>
+        </is>
+      </c>
+      <c r="B86">
+        <v>14</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>ELMo (Embeddings from Language Models) is a pre‑trained contextual word embedding model that can be fine‑tuned for tasks such as sentiment or opinion analysis, but it was not created specifically for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>PSO</t>
+        </is>
+      </c>
+      <c r="B87">
+        <v>14</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>PSO (Particle Swarm Optimization) is a general-purpose optimization algorithm; it is not a software tool for extracting opinions and is not specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Apache Hadoop MapReduce</t>
+        </is>
+      </c>
+      <c r="B88">
+        <v>13</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Apache Hadoop MapReduce is a distributed computing framework for processing large data sets; it can support opinion‑measurement pipelines but is not itself a tool for extracting opinions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>CNN-BiLSTM</t>
+        </is>
+      </c>
+      <c r="B89">
+        <v>13</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>CNN‑BiLSTM is a neural network architecture combining convolutional layers with a bidirectional LSTM, commonly used for text classification tasks such as sentiment or opinion analysis, but it is a generic algorithm rather than a dedicated opinion‑measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Google Cloud Natural Language API</t>
+        </is>
+      </c>
+      <c r="B90">
+        <v>13</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>commercial_api</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Google Cloud Natural Language API is a proprietary cloud service offering NLP functions such as sentiment analysis, entity sentiment, and text classification, enabling extraction of opinions from text; sentiment analysis is a core feature, making it specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>NTUSD</t>
+        </is>
+      </c>
+      <c r="B91">
+        <v>13</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>linguistic_resource</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>NTUSD (National Taiwan University Sentiment Dictionary) is a lexical resource providing sentiment scores for Chinese words, designed specifically for sentiment and opinion analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="B92">
+        <v>13</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>T5 (Text‑to‑Text Transfer Transformer) is a pre‑trained transformer model that can be fine‑tuned for many NLP tasks, including sentiment or opinion analysis, but it is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>XLM-RoBERTa</t>
+        </is>
+      </c>
+      <c r="B93">
+        <v>13</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>XLM-RoBERTa is a pre‑trained multilingual transformer model that can be fine‑tuned for various NLP tasks, including sentiment or opinion analysis, but it is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>GCN</t>
+        </is>
+      </c>
+      <c r="B94">
+        <v>12</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>GCN (Graph Convolutional Network) is a general neural network architecture for learning on graph-structured data; it can be applied to opinion/sentiment tasks but is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>MeaningCloud</t>
+        </is>
+      </c>
+      <c r="B95">
+        <v>12</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>commercial_api</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>MeaningCloud is a commercial cloud‑based API that offers text analytics services such as sentiment and opinion analysis, making it directly usable for measuring opinions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Stanford POS Tagger</t>
+        </is>
+      </c>
+      <c r="B96">
+        <v>12</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>single_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>The Stanford POS Tagger is a dedicated tool for part‑of‑speech tagging of text, useful for linguistic preprocessing but not designed to measure opinions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>TC-LSTM</t>
+        </is>
+      </c>
+      <c r="B97">
+        <v>12</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>TC-LSTM (Target‑Conditioned LSTM) is a neural network architecture designed for aspect‑based sentiment analysis, enabling opinion measurement toward specific targets. It is an algorithmic model rather than a packaged software tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ASUM</t>
+        </is>
+      </c>
+      <c r="B98">
+        <v>11</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>ASUM (Aspect and Sentiment Unification Model) is a pre‑trained probabilistic model for joint aspect extraction and sentiment analysis, specifically designed for opinion measurement, but it is typically described in research papers rather than released as a reusable software package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>AT-LSTM</t>
+        </is>
+      </c>
+      <c r="B99">
+        <v>11</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>AT-LSTM is an attention‑based LSTM architecture proposed for aspect‑level sentiment (opinion) analysis; it can be used to measure opinions but is primarily a model design rather than a packaged software tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Apache OpenNLP</t>
+        </is>
+      </c>
+      <c r="B100">
+        <v>11</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>general_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Apache OpenNLP is an open‑source Java library offering a range of NLP components (tokenizer, POS tagger, NER, etc.) that can be employed to build opinion/sentiment analysis pipelines, though it is not specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Attention-BiLSTM</t>
+        </is>
+      </c>
+      <c r="B101">
+        <v>11</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Attention‑BiLSTM is a neural network architecture (bidirectional LSTM with an attention mechanism) that can be applied to tasks like sentiment or opinion analysis, but it is a general method rather than a dedicated opinion‑measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Bayesian Network</t>
+        </is>
+      </c>
+      <c r="B102">
+        <v>11</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>A probabilistic graphical model used for reasoning under uncertainty; it can be applied to opinion/sentiment classification tasks but is not a tool specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>DCNN</t>
+        </is>
+      </c>
+      <c r="B103">
+        <v>11</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>DCNN (Deep Convolutional Neural Network) is a neural network architecture that can be applied to many text classification tasks, including sentiment or opinion analysis, but it is not itself a dedicated opinion measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>DistilBERT</t>
+        </is>
+      </c>
+      <c r="B104">
+        <v>11</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>DistilBERT is a pre‑trained, distilled transformer language model that can be fine‑tuned for tasks such as sentiment or opinion analysis, but it is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Gaussian Naive Bayes</t>
+        </is>
+      </c>
+      <c r="B105">
+        <v>11</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Gaussian Naive Bayes is a probabilistic classification algorithm that can be applied to sentiment or opinion classification tasks, but it is a general machine‑learning method, not a dedicated opinion‑measurement tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="B106">
+        <v>11</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Hidden Markov Model (HMM) is a statistical sequence modeling algorithm that can be applied to tasks like sentiment or opinion analysis, but it is a general algorithm not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>NVivo</t>
+        </is>
+      </c>
+      <c r="B107">
+        <v>11</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>gui_tool</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>NVivo is a commercial qualitative data analysis desktop application with a graphical user interface that supports coding and analysis of textual data, allowing researchers to examine opinions and sentiments, though it is not specifically built for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>SnowNLP</t>
+        </is>
+      </c>
+      <c r="B108">
+        <v>11</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>general_purpose_nlp</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>SnowNLP is a Python library for Chinese text processing that provides functions such as sentiment analysis, text classification, and keyword extraction; it can be used for opinion measurement but is not dedicated solely to that purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>TensorFlow</t>
+        </is>
+      </c>
+      <c r="B109">
+        <v>11</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>general_library</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>TensorFlow is an open‑source machine learning framework that can be used to build models for many tasks, including opinion/sentiment analysis, but it is not specifically designed for opinion measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>n-gram</t>
+        </is>
+      </c>
+      <c r="B110">
+        <v>11</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>approach</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>n‑gram is a textual representation technique (e.g., unigrams, bigrams) used in many NLP models, including sentiment and opinion analysis, but it is a methodological concept rather than a specific software tool.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>